<commit_message>
feat: el motor cobra por folio y envejece por partida
</commit_message>
<xml_diff>
--- a/docs/DEMO_Agrodrones_Bajio_FICTICIO.xlsx
+++ b/docs/DEMO_Agrodrones_Bajio_FICTICIO.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="878" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="344">
   <si>
     <t xml:space="preserve">ARCHIVO DE DEMOSTRACION — DATOS COMPLETAMENTE FICTICIOS</t>
   </si>
@@ -2233,17 +2233,17 @@
       </c>
       <c r="P10" s="15" t="n">
         <f aca="false">IFERROR(SUMIF(cobranza!$B$3:$B$1000,A10,cobranza!$D$3:$D$1000),0)</f>
-        <v>100000</v>
+        <v>124000</v>
       </c>
       <c r="Q10" s="15" t="n">
         <f aca="false">IFERROR(H10-P10,"")</f>
-        <v>165000</v>
+        <v>141000</v>
       </c>
       <c r="R10" s="17"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B11" s="12" t="n">
         <v>46119</v>
@@ -2271,9 +2271,7 @@
         <v>47</v>
       </c>
       <c r="K11" s="11"/>
-      <c r="L11" s="11" t="s">
-        <v>58</v>
-      </c>
+      <c r="L11" s="11"/>
       <c r="M11" s="11" t="s">
         <v>48</v>
       </c>
@@ -2287,11 +2285,11 @@
       </c>
       <c r="P11" s="15" t="n">
         <f aca="false">IFERROR(SUMIF(cobranza!$B$3:$B$1000,A11,cobranza!$D$3:$D$1000),0)</f>
-        <v>24000</v>
+        <v>124000</v>
       </c>
       <c r="Q11" s="15" t="n">
         <f aca="false">IFERROR(H11-P11,"")</f>
-        <v>0</v>
+        <v>-100000</v>
       </c>
       <c r="R11" s="17"/>
     </row>
@@ -2615,17 +2613,17 @@
       </c>
       <c r="P17" s="15" t="n">
         <f aca="false">IFERROR(SUMIF(cobranza!$B$3:$B$1000,A17,cobranza!$D$3:$D$1000),0)</f>
-        <v>420000</v>
+        <v>431500</v>
       </c>
       <c r="Q17" s="15" t="n">
         <f aca="false">IFERROR(H17-P17,"")</f>
-        <v>100000</v>
+        <v>88500</v>
       </c>
       <c r="R17" s="17"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B18" s="12" t="n">
         <v>46205</v>
@@ -2669,11 +2667,11 @@
       </c>
       <c r="P18" s="15" t="n">
         <f aca="false">IFERROR(SUMIF(cobranza!$B$3:$B$1000,A18,cobranza!$D$3:$D$1000),0)</f>
-        <v>11500</v>
+        <v>431500</v>
       </c>
       <c r="Q18" s="15" t="n">
         <f aca="false">IFERROR(H18-P18,"")</f>
-        <v>0</v>
+        <v>-420000</v>
       </c>
       <c r="R18" s="17"/>
     </row>
@@ -12241,7 +12239,7 @@
         <v>141</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C14" s="12" t="n">
         <v>46119</v>
@@ -12430,7 +12428,7 @@
         <v>151</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C23" s="12" t="n">
         <v>46205</v>

</xml_diff>

<commit_message>
fix: el aviso de días de crédito solo sale con saldo, y la hoja ausente es advertencia
</commit_message>
<xml_diff>
--- a/docs/DEMO_Agrodrones_Bajio_FICTICIO.xlsx
+++ b/docs/DEMO_Agrodrones_Bajio_FICTICIO.xlsx
@@ -1570,7 +1570,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:B17"/>
+  <dimension ref="B2:B26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="100"/>
@@ -1646,6 +1646,62 @@
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="2" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Dos ventas con varios productos en el mismo folio (V-008 y V-015).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Avisos que vera al cargar este archivo. Ninguno es un error: estan puestos a proposito.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Linea Demo (V-006): es una unidad de exhibicion, no una venta. Se lista aparte y no cuenta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Abonos que suman mas que el precio (V-018): se cobro de mas, para mostrar un saldo a favor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Falta fecha (V-025): una venta sin fecha de entrega. Se reporta aparte, no se descarta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Condicion distinta en sus partidas (V-015): el equipo dice Credito y su accesorio Contado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    La aplicacion aplica el primero a toda la venta y lo avisa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Sin dias de credito y con saldo (cinco ventas): su antiguedad se mide desde la entrega.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>